<commit_message>
Rebuild lead list with corrected parcel dataset
Uses the full pqrn-qghw export (real state_use_description column),
so candidate parcels now rank by actual use codes
(commercial/apartment above single-family).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eb8pFNbEASzxnuWc7CqGLH
</commit_message>
<xml_diff>
--- a/cttowerleads/ct-tower-leads/output/leads.xlsx
+++ b/cttowerleads/ct-tower-leads/output/leads.xlsx
@@ -584,7 +584,11 @@
           <t>HENNESSEY SHARON M; QUIROS  MARGARET R TRUST; QUIROS MARGARET R TRUST; SINGER CLAUDE</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>ONE FAMILY; VAC UNDV RES; VAC LAND RES; AUX IMP RES</t>
+        </is>
+      </c>
       <c r="J5" s="4" t="n">
         <v>38</v>
       </c>
@@ -620,15 +624,19 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>177 RETREAT AVE; 179 RETREAT AVE; 195 RETREAT AVE; 199 RETREAT AVE</t>
+          <t>140 RETREAT AVE; 136 RETREAT AVE; 179 RETREAT AVE; 177 RETREAT AVE</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>HARTFORD HOSPITAL; INSTITUTE OF LIVING; HARTFORD HOSPITAL; CIL REALTY INC</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="n"/>
+          <t>HARTFORD HOSPITAL; HARTFORD HOSPITAL; CENTURION HOLDINGS 1 INC; HARTFORD HOSPITAL</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>MED OFFICE; MED OFFICE; MED OFFICE; GEN HOSPITAL</t>
+        </is>
+      </c>
       <c r="J6" s="4" t="n">
         <v>20</v>
       </c>
@@ -674,7 +682,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Commercial Building; Commercial Building; Commercial Building; Commercial Apt 5+ units</t>
+          <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Apt</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
@@ -712,15 +720,19 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>110 PECK ST; 106 PECK ST; 102 PECK ST; 200 PECK ST</t>
+          <t>319 PECK ST; 110 PECK ST; 106 PECK ST; 102 PECK ST</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>MASSARO PROPERTIES LLC; HAYWARD MAGDALIA; VANDERPOOL LARRY; DEFRANCESCO MARK &amp; LAUREN</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="n"/>
+          <t>ERECTOR SQUARE LLC; MASSARO PROPERTIES LLC; HAYWARD MAGDALIA; VANDERPOOL LARRY</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>INDUSTRIAL  MDL-96; Three Family; Two Family; Three Family</t>
+        </is>
+      </c>
       <c r="J8" s="4" t="n">
         <v>64</v>
       </c>
@@ -752,17 +764,17 @@
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>150 WHALLEY AV; 116 WHALLEY AV; 193 WHALLEY AV; 101 WHALLEY AV</t>
+          <t>157 WHALLEY AV; 223 WHALLEY AV; 292 WHALLEY AV; 208 WHALLEY AV</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>CORAL NEW HAVEN ASSOCIATES II*; U HAUL REAL ESTATE CO; HEER REAL ESTATE LLC; 101 WHALLEY LLC</t>
+          <t>VECE PROPERTIES LLC; HUTT DAVID; D J M ENTERPRISES INC; MAHAS PROPERTIES LLC</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>(INC/MKT ADJ); APP W/01900</t>
+          <t>COMM WHSE  MDL-95; OFFICE BLD  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
@@ -800,17 +812,17 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>28 RICHARDS AVE; 15 RICHARDS AVE; 93 RICHARDS AVE; 75 RICHARDS AVE</t>
+          <t>93 RICHARDS AVE; 75 RICHARDS AVE; 40 RICHARDS AVE; 50 RICHARDS AVE</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>DEORIO VINCENT J TRUSTEE OF THE; FURNAROS RICHARD M &amp; CHARLOTTE; 93 RICHARDS REALTY I LLC 83% &amp;; NEW ENGLAND HOLDINGS II</t>
+          <t>93 RICHARDS REALTY I LLC 83% &amp;; NEW ENGLAND HOLDINGS II; 40 RICHARDS LLC; NORWALKIN LLC</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>MED TRAFFIC; HWYADJ; COMM INFL; COMM INFL; MED TRAFFIC; OFF CON AVE</t>
+          <t>Apartments - Com; Commercial Improved; Commercial Improved; Commercial Improved</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
@@ -848,17 +860,17 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>25 BELDEN AVE; 11 BELDEN AVE; 17 BELDEN AVE; 15 BELDEN AVE</t>
+          <t>25 BELDEN AVE; 11 BELDEN AVE; 30 BELDEN AVE; 24 BELDEN AVE</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>DEPANFILIS ANTHONY J; NORWALK CITY OF; CONNECTICUT STATE OF; 587 BELDEN LLC</t>
+          <t>DEPANFILIS ANTHONY J; NORWALK CITY OF; BELDEN HOLDING COMPANY LLC; RITZ REALTY CORP</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>OFF WEST AVE</t>
+          <t>Commercial Improved; Commercial Improved; Commercial Improved; Commercial Improved</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
@@ -926,15 +938,19 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>275 WINDSOR ST; 300 WINDSOR ST; 150 WINDSOR ST; 847 WINDSOR ST</t>
+          <t>275 WINDSOR ST; 300 WINDSOR ST; 835 WINDSOR ST; 716 WINDSOR ST</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>RMS 275 WINDSOR STREET LLC; TRAVELERS INDEMNITY CO; CITY OF HARTFORD; 847 WINDSOR STREET LLC</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n"/>
+          <t>RMS 275 WINDSOR STREET LLC; TRAVELERS INDEMNITY CO; CONN LIGHT &amp; POWER CO; 716 WINDSOR PROPERTIES LLC</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>GEN OFFICE; GEN OFFICE; AUX IMP COMM; GEN OFFICE</t>
+        </is>
+      </c>
       <c r="J13" s="6" t="n">
         <v>52</v>
       </c>
@@ -978,7 +994,11 @@
           <t>STATE OF CONN ADRIAEN`S LANDING; CHILIDOG50C LLC; CONN NATURAL GAS CORP; ENERGY NETWORKS INC</t>
         </is>
       </c>
-      <c r="I14" s="7" t="n"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>ST-ADMINISTR; HIGH RISE OF; OTHER UTILTY; A PARKING</t>
+        </is>
+      </c>
       <c r="J14" s="6" t="n">
         <v>26</v>
       </c>
@@ -1024,7 +1044,7 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Commercial Building; Commercial Building; Commercial Building; Commercial Land</t>
+          <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Land</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
@@ -1058,15 +1078,19 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>34 SHELTON AV; 62 SHELTON AV; 60 SHELTON AV; 58 SHELTON AV</t>
+          <t>13 SHELTON AV; 99 SHELTON AV; 89 SHELTON AV; 34 SHELTON AV</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>BAILEY SHERRY J; DAGAN ROCHELL TR; DANNY GUY 3 DE LLC; 1423 Q 811 LLC</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="n"/>
+          <t>HS SHELTON LLC; BLUE BAHIA PROPERTIES LLC; NEW HAVEN BUSINESS CENTER LLC; BAILEY SHERRY J</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; INDUSTRIAL  MDL-96; INDUSTRIAL  MDL-96; Two Family</t>
+        </is>
+      </c>
       <c r="J16" s="6" t="n">
         <v>147</v>
       </c>
@@ -1102,15 +1126,19 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>584 PROSPECT ST; 648 PROSPECT ST; 314 PROSPECT ST; 310 PROSPECT ST</t>
+          <t>400 PROSPECT ST; 584 PROSPECT ST; 648 PROSPECT ST; 314 PROSPECT ST</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>D &amp; L MANCHESTER LLC; BORELLINI VICTOR E JR; YALE UNIVERSITY; YALE UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="n"/>
+          <t>YALE UNIVERSITY; D &amp; L MANCHESTER LLC; BORELLINI VICTOR E JR; YALE UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>OFFICE BLD  MDL-94; APT5 - 12 R  MDL-03; Single Family; PVT UNIV  MDL-94</t>
+        </is>
+      </c>
       <c r="J17" s="6" t="n">
         <v>59</v>
       </c>
@@ -1142,17 +1170,17 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>1040 WHALLEY AV; 1226 WHALLEY AV; 1222 WHALLEY AV; 1218 WHALLEY AV</t>
+          <t>1190 WHALLEY AV; 1297 WHALLEY AV; 1307 WHALLEY AV; 1045 WHALLEY AV</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>CHAPEL HAVEN SCHLEIFER CENTER; NETZ KEREN DE LLC; STAFFORD SAMUEL; CHIAL LLC</t>
+          <t>ONOFRIO BIAGIO &amp; ANNA MARIA; DIRIENZO ENTERPRISES LLC; SINGHANARATHA KANYANEE; SMART HOUSE LLC</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>ALL SITE; COND = TOPO; LOC 3</t>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; OFFICE BLD  MDL-94</t>
         </is>
       </c>
       <c r="J18" s="6" t="n">
@@ -1186,17 +1214,17 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>196 CHAPEL ST; 184 CHAPEL ST; 178 CHAPEL ST; 168 CHAPEL ST</t>
+          <t>178 CHAPEL ST; 166 CHAPEL ST; 153 CHAPEL ST; 159 CHAPEL ST</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>LLOYD-CHAPEL LLC; LLOYD-CHAPEL LLC; 178 CHAPEL STREET ASSOCIATES LLC; 178 CHAPEL STREET LLC</t>
+          <t>178 CHAPEL STREET ASSOCIATES LLC; ART CT 770 LAND LLC; SZE REALTY LLC; SPERRY GROUP DE2 LLC</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>SITE; W/PID 8099; W/PID 8098</t>
+          <t>INDUSTRIAL  MDL-96; INDUSTRIAL  MDL-96; COMM WHSE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
       <c r="J19" s="6" t="n">
@@ -1240,7 +1268,7 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>W/PID 184008; WITH LIST 001-3793</t>
+          <t>Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94; Commercial  MDL-00</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
@@ -1274,15 +1302,19 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>70 KNAPP STREET; 88 KNAPP STREET; 74 KNAPP STREET; 93 KNAPP STREET</t>
+          <t>22 KNAPP STREET; 18 KNAPP STREET; 70 KNAPP STREET; 88 KNAPP STREET</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>DESOUSA NELSON A ET AL; HUNT BRIAN ET AL; JOELSON DAVID F ET AL; BORDA EDDY ET AL</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="n"/>
+          <t>YB WORLD LLC; KNAPP ST INVESTORS; DESOUSA NELSON A ET AL; HUNT BRIAN ET AL</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Apartment  MDL-94; Single Family; Single Family</t>
+        </is>
+      </c>
       <c r="J21" s="6" t="n">
         <v>31</v>
       </c>
@@ -1318,15 +1350,19 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>61 SEAVIEW AVENUE; 61 SEAVIEW AVENUE; 61 SEAVIEW AVENUE; 61 SEAVIEW AVENUE</t>
+          <t>43 SEAVIEW AVENUE; 68 SEAVIEW AVENUE; 23 SEAVIEW AVENUE; 61 SEAVIEW AVENUE</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>TAM PETER ET AL; REEVES BRENDAN; FREYER CHRISTIAN ET AL; BEDNARCZYK SOPHIE</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="n"/>
+          <t>MOORINGS APARTMENTS INC; SEAVIEW HOUSE LLC; 23 SEAVIEW STAMFORD LLC; TAM PETER ET AL</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>Apartment  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Res. Condo</t>
+        </is>
+      </c>
       <c r="J22" s="6" t="n">
         <v>85</v>
       </c>
@@ -1368,7 +1404,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Commercial Building; Industrial Building; Residential Improved; Residential Improved</t>
+          <t>Comm Bldg; Ind Bldg; Res Impr; Res Impr</t>
         </is>
       </c>
       <c r="J23" s="6" t="n">

</xml_diff>

<commit_message>
Include single-carrier sites in lead list (min-active=1)
Lowers the active-carrier threshold from 2 to 1: 79 leads total
(60 with 1 active carrier, 12 with 2, 7 gold with 3+).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eb8pFNbEASzxnuWc7CqGLH
</commit_message>
<xml_diff>
--- a/cttowerleads/ct-tower-leads/output/leads.xlsx
+++ b/cttowerleads/ct-tower-leads/output/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$4:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$4:$J$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1411,8 +1411,2588 @@
         <v>90</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>*** Wordin Avenue</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>750 WORDIN AV; 276 WORDIN AV; 129 WORDIN AV; 299 WORDIN AV</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>GEDNEY MARY LOUISE; CONNECTICUT RESOURCES; 129 WORDIN AVENUE LLC; PS PROPERTIES ADVISORS INC</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Industrial Mdl 96; Industrial Lnd; Industrial Mdl 96; Self Storage</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>*** Arctic Street</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>211 ARCTIC ST; 227 ARCTIC ST; 138 ARCTIC ST; 108 ARCTIC ST</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>CATALAN ERIK L G; D &amp;F PROPERTY MANAGEMENT LLC; OGARRO PETER G &amp; DENISE; MIAKOS NICHOLAS</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Two Family; Single Family; Single Family; Two Family</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>**** North Avenue</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Nextel→TMO?</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>1123 NORTH AV; 1207 NORTH AV; 1215 NORTH AV; 1375 NORTH AV</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>AEA MGMT LLC; ARBER MANAGEMENT LLC; ARBER MANAGEMENT LLC; WEBSTER SCHOOL REALTY LLC</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Mix Use Comm; Comm Apts; Mix Use Comm; Comm Apts</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>*** Park Avenue (*** University Ave.)</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>538 PARK AV; 500 PARK AV; 448 PARK AV; 378 PARK AV</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>ARROYO HECTOR; 500 PARK AVE CORP; COLMENA PROPERTIES LLC; BATH GURVINDER</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Mix Use Comm; Retail Strip/Plaza; Comm Apts; Mix Use Comm</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>*** Grant Street</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>445 GRANT ST; 540 GRANT ST; 267 GRANT ST; 267 GRANT ST</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>GRANT PROPERTY GROUP LLC; SLC 540 GRANT ST LLC; BRIDGEPORT HOSPITAL; BRIDGEPORT HOSPITAL</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Industrial Mdl 96; Industrial Mdl 96; Hospital; Hospital</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Bridgeport</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>*** Newfield Avenue</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>billboard</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>549 NEWFIELD AV; 193 NEWFIELD AV; 568 NEWFIELD AV; 101 NEWFIELD AV</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>HIGHLAND STREET ASSOCATES; TAVERAS RUDIS; H G STRATFORD ASSOCIATES LLC; VILLAR IRIS</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Vac Comm Lnd; Mix Use Comm; Comm Apts; Single Family</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>**** Main Sreet</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>rooftop small cell</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+      <c r="J30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>*** Main Street</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>330 MAIN ST; 990 MAIN ST; 19-29 MAIN ST; 197 MAIN ST</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>SGS 330 MAIN LLC; PCX 990 LLC; MIND EQUITIES LLC; CITY OF HARTFORD FIRE DEPT</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>GEN OFFICE; RETAIL GEN; GEN OFFICE; CITY-FIRE</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>*** Woodland Street</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>433 WOODLAND ST; 103 WOODLAND ST; 148 WOODLAND ST; 359 WOODLAND ST</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>ASSET 10305 LLC; BRIDGETOWN LLC; 148-150 WOODLAND ST LLC; M&amp;EM REALTY LLC</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>GEN OFFICE; MED OFFICE; RETAIL GEN; APARTMENT</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>*** Summit Street</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>rooftop/faux chimney</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>340 SUMMIT ST; 340 SUMMIT ST; 260 SUMMIT ST; 451-453 SUMMIT ST</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>ST ANTHONY HALL FOUNDATION; ST ANTHONY HALL FOUNDATION; TRINITY COLLEGE TRUSTEES OF; OCORO MIREYA</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>CHARITABLE; HALL - CLUB; PRIV COLLEGE; THREE FAMILY</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>** Sigourney Street</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>25 SIGOURNEY ST; 45 SIGOURNEY ST; 35 SIGOURNEY ST; 85 SIGOURNEY ST</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>SPARTAN TOWERS LLC; STATE OF CONN DEPT OF TRANS; STATE OF CONN; 85 SIGOURNEY HOLDING LLC</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>HIGH RISE OF; ST-DOT; ST-MISC PROP; HIGH RISE OF</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>** Trumbull St</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>building mount</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>140-150 TRUMBULL ST; 55 TRUMBULL ST; 34-36 TRUMBULL ST; 218-260 TRUMBULL ST</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>SGS 150 TRUMBULL LLC; 55 TRUMBULL STREET ASSOC; CARA HOLDINGS INC; SHELBOURNE PRATT DEVELOPMENT LLC</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>GEN OFFICE; APT HIGH RSE; GEN OFFICE; HIGH RISE OF</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>**** Main Street (** New Donald St)</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>1325 MAIN ST; 1491 MAIN ST; 2087 MAIN ST; 2279 MAIN ST</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>527 MAIN STREET PROPERTIES LLC; MCDONALD MONICA; MARTIN JOY A; THOMAS GARIE</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>APART/COMM; RETAIL GEN; RES/COMM; RES/COMM</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>*** Asylum Street</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>building mount</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>518 ASYLUM ST; 525 ASYLUM ST; 402-418 ASYLUM ST; 309 ASYLUM ST</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>STATE OF CONN DEPT OF TRANS; STATE OF CONN HIGHWAY DEPT; 410 ASYLUM STREET LLC; P S C DEVELOPMENT LLC</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>ST-MISC PROP; ST-HWY PROP; APART/COMM; L PARKING</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>*** Prospect Avenue</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>100 PROSPECT AVE; 112 PROSPECT AVE; 340 PROSPECT AVE; 408 PROSPECT AVE</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>7HART LLC; 112 PROSPECT AVE REALTY LLC; 2074-2100 PARK STREET LLC; HEARTHSTONE PROSPECT AVENUE LLC</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>APARTMENT; GEN OFFICE; RETAIL GEN; APARTMENT</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>*** Sisson Avenue</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>227 SISSON AVE; 137 SISSON AVE; 252 SISSON AVE; 91-99 SISSON AVE</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>JIMINIAN CRISTOBAL; GHAMO PROPERTIES LLC; 252 SISSON LLC; BOTTOMS UP LLC</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>RES/COMM; RETAIL GEN; APARTMENT; APART/COMM</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>* State St</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>building mount</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>0 STATE ST; 0 STATE ST; 0 STATE ST; 50-58 STATE ST</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>TK STATE HOUSE LLC; TK STATE HOUSE LLC; TK STATE HOUSE LLC; MAC-STATE SQUARE LLC</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>VAC LAND COM; VAC LAND COM; VAC LAND COM; HIGH RISE OF</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>**** Park Street</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>smokestack</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>1870 PARK ST; 1840 PARK ST; 1850 PARK ST; 1814 PARK ST</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>BARBOSA DOMINGOS D; 1840 PARK LLC; NGUYEN HAI H; 1814 PARK ST LLC</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>RES/COMM; RETAIL GEN; RETAIL GEN; COMM &amp; APART</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>*** Garden Street</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>665 GARDEN ST; 195 GARDEN ST; 140 GARDEN ST; 225 GARDEN ST</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>SPIN GHAR PROPERTIES LLC; YOUNG WOMENS CHRISTIAN ASSOC OF THE HTFD REGION INC; HLA LLC; FAUST LAWRENCE</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>APARTMENT; CHARITABLE; HIGH RISE OF; ONE FAMILY</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>*** Bartholomew Avenue</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>136 BARTHOLOMEW AVE; 132-134 BARTHOLOMEW AVE; 175 BARTHOLOMEW AVE; 169 BARTHOLOMEW AVE</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>ALVARENGA MONICA A; JYB LLC; 237 HAMILTON I L L C; RGH BARTHOLOMEW LLC</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>ONE FAMILY; APARTMENT; VAC LAND IND; MANUFACTURNG</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>*** Maple Avenue</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>895 MAPLE AVE; 901 MAPLE AVE; 871 MAPLE AVE; 944 MAPLE AVE</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>ROCHA RIORDAN; MAPLE AVENUE LAUNDOMAT LLC; PAYAL LLC; GEORGERAYMOND REAL ESTATE &amp; INVESTMENTS LLC</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>AUX IMP COMM; RETAIL GEN; RETAIL GEN; RETAIL GEN</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>** Woodland Street</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>21 WOODLAND ST; 43 WOODLAND ST; 95 WOODLAND ST; 36 WOODLAND ST</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>WOODLAND STREET LLC; WHEELER CLINIC INC; ST FRANCIS HOSPITAL &amp; MEDICAL CENTER; WOODLAND 36 LLC</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>MED OFFICE; MED OFFICE; MED OFFICE; GEN OFFICE</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>** Webster Street</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>MetroPCS→TMO?</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>56 WEBSTER ST; 90 WEBSTER ST; 97 WEBSTER ST; 89 WEBSTER ST</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>ETERNAL ENTERPRISE INC; 90 WEBSTER STREET TOWER LLC; MELIUS STEVIE; CHRYSALIS CENTER REAL ESTATE CORPORATION</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>APARTMENT; APARTMENT; ONE FAMILY; CHARITABLE</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>** Farmington Avenue</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>86 FARMINGTON AVE; 527-535 FARMINGTON AVE; 509-511 FARMINGTON AVE; 505-507 FARMINGTON AVE</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>86 FARMINGTON AVENUE ASSOC LLC; ELLIS JONES ALTHEA; PERFITO NICHOLAS V; PERFITO NICHOLAS J</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>GEN OFFICE; APART/COMM; RES/COMM; COMM/RES</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>** Elliott Street</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>22 ELLIOTT ST; 50 ELLIOTT ST; 52 ELLIOTT ST; 49 ELLIOTT ST</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>280H LLC; JESS PROPERTIES LLC; ELLIOTT 52 STREET LLC; OWEN INVESTMENTS LLC</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>APARTMENT; APARTMENT; APARTMENT; THREE FAMILY</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Hartford</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>*** Brainard Road</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>smokestack</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>167 BRAINARD RD; 160 BRAINARD RD; 100 BRAINARD RD; 255 BRAINARD RD</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>167 BRAINARD RD LLC; D &amp; C FAMILY LLC; DFC LLC; THE METROPOLITAN DISTRICT</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>RETAIL GEN; RETAIL GEN; RETAIL GEN; SPECIAL ACTS</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>*** Chamberlain Highway</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>133 CHAMBERLAIN HWY; 190 CHAMBERLAIN HWY; 474 CHAMBERLAIN HWY; 261 CHAMBERLAIN HWY</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>NOOR 12 LLC; ARBOR I LLC; TARGET CORPORATION; CHAMBERLAIN HEIGHTS</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>Comm Bldg; Comm Apt; Comm Bldg; Comm Apt</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>***-*** East Main Street</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>783 EAST MAIN ST; 725 EAST MAIN ST; 722 EAST MAIN ST; 113 EAST MAIN ST</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>MCDONALDS CORP; KATE FRANK 725 EAST MAIN STREE; VICTORY MERIDEN REALTY LLC; 113 E MAIN LLC</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Apt</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>*** South Broad Street</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>smokestack</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Sprint→TMO?, Nextel→TMO?, MetroPCS→TMO?</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="n"/>
+      <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
+      <c r="J52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>** Willow Street</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>Nextel→TMO?</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>90 WILLOW ST; 82 WILLOW ST; 40 WILLOW ST; 24 WILLOW ST</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>ST MARYS GERMAN HERITAGE SOCIETY INC; PELLOT ALEX JAIME; PRIME INVESTMENTS LLC; GALINDO ISRAEL GONZALEZ</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>Comm Bldg; Res Impr; Vacant Com; Res Impr</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>**** East Main Street</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>1260 EAST MAIN ST; 1239 EAST MAIN ST; 1333 EAST MAIN ST; 1544 EAST MAIN ST</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>MWT PROPERTIES LLC; TWELVE FIFTY SEVEN EAST MAIN S; YUM LINDA; 94 WARNER ASSOCIATES LLC</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Land</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>*** Pratt Street</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>234 PRATT ST; 135 PRATT ST; 256 PRATT ST; 145 PRATT ST</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>TORRES ELVIN &amp;; CARABETTA ENTERPRISES INC; CHEHOTSKY STEVEN; PRATT &amp; TWISS ST LLC</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>Comm Bldg; Comm Land; Comm Bldg; Comm Land</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>** Water Street</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>Nextel→TMO?</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>26 WATER ST; 83 WATER ST; 89 WATER ST; 99 WATER ST</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>MACKENZIE KENNETH H JR; AMERCO REAL ESTATE COMPANY; P H K P ASSOCIATES INC; BROWN STREET NEW HAVEN LLC</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>INDUSTRIAL  MDL-96; IND WHSES  MDL-96; REST/CLUBS  MDL-94; PARK LOT</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>** Whalley Avenue</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>MetroPCS→TMO?</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>14 WHALLEY AV; 43 WHALLEY AV; 53 WHALLEY AV; 30 WHALLEY AV</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>14 16 18 WHALLEY AVENUE LLC; YALE UNIVERSITY; LEW LEHRER FAMILY TRUST; SUMMIT HOSPITALITY 145 LLC</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; HOTELS  MDL-94</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="n">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>** McKinley Avenue</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>in-building IP access</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>90 MCKINLEY AV; 84 MCKINLEY AV; 76 MCKINLEY AV; 70 MCKINLEY AV</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>SCHWARTZ RONALD J; MORRIS COHEN TR &amp; GLORIA COHEN*; BURCHELL IAIN; ACOCELLA PATRICIA &amp; STOLLERMAN SANDY</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>Single Family; Single Family; Single Family; Single Family</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>*** Orange Street</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>794 ORANGE ST; 829 ORANGE ST; 528 ORANGE ST; 494 ORANGE ST</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>DIPAOLA MARK PETER; TIDEWAYS EAST LLC; PEARL ON ORANGE LLC; CIANCIOLO PROPERTIES LLC</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>*** Howard Avenue</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>529 HOWARD AV; 399 HOWARD AV; 407 HOWARD AV; 485 HOWARD AV</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>RITAD LLC; NHCD 8 LLC; BBYM DE2 LLC; 485-487 HOWARD AVE INC</t>
+        </is>
+      </c>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>*** Forbes St.</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>building mount</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="7" t="n"/>
+      <c r="H61" s="7" t="n"/>
+      <c r="I61" s="7" t="n"/>
+      <c r="J61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>*** College Street</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>265 COLLEGE ST; 268 COLLEGE ST; 266 COLLEGE ST; 260 COLLEGE ST</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>PAR TAFT LLC; 268 COLLEGE STREET LLC; FORK 266 COLLEGE LLC; YALE UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>*** Pond Lily Avenue</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>billboard</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>140 POND LILY AV; 100 POND LILY AV; 105 POND LILY AV; 111 POND LILY AV</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>STATE OF CONNECTICUT; A &amp; C REALTY LLC; WALLER WILLIAM &amp; GAIL; MOORE CARLTON &amp; JEWEL A</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>STATE DOT  MDL-95; MOTELS; Single Family; Single Family</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>*** N. Frontage Road</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="7" t="n"/>
+      <c r="H64" s="7" t="n"/>
+      <c r="I64" s="7" t="n"/>
+      <c r="J64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>** Warren Street</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>49 WARREN ST; 55 WARREN ST; 63 WARREN ST; 67 WARREN ST</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>REF II SFR 1 DE LLC; DANA MAISON DE POUPEE LLC &amp;; SCARPELLINO ANGIE; TIBONI JACK E</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>APT 4-Unit; APT5 - 12  MDL-94; Three Family; Three Family</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>*** Winchester Avenue</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>275 WINCHESTER AV; 597 WINCHESTER AV; 265 WINCHESTER AV; 518 WINCHESTER AV</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>SPDC TRACT A LLC; RODRIGUEZ JOSE; YIK VINCENT; LIVINGSTON LARRY</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>INDUSTRIAL  MDL-96; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
+        </is>
+      </c>
+      <c r="J66" s="6" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>*** State Street</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>957 STATE ST; 965 STATE ST; 969 STATE ST; 973 STATE ST</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>STATE PROPERTY MANAGEMENT*; 965 STATE LLC; RBA ASSOCIATES; 5 WEST MAIN STREET LLC</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Norwalk</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>* Selleck Street</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="n"/>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>1 SELLECK ST; 2 SELLECK ST; 6 SELLECK ST; 4 SELLECK ST</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>AMERCO REAL ESTATE COMPANY; SOLDER WILLIAM &amp; DONNA M; BAILEY SANDRA; MATHEWS GEORGE E</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Improved; 3 Family; Single Family; 2 Family</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>Norwalk</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>** Day Street</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n"/>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>19 DAY ST; 17 DAY ST; 11 DAY ST; 20 DAY ST</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>ALPHA5MK 19 DAY LLC; SONO SQUARE ASSOCIATES LLC 25% &amp;; IBI LLC; HOUSING AUTHORITY-CITY OF NORWALK-LESSOR</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Improved; Commercial Vacant; Commercial Improved; Apartments - Com</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Norwalk</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>*** Main Avenue (** Glover Avenue)</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>rooftop/in-building</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n"/>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>280 MAIN AVE; 300 MAIN AVE; 306 MAIN AVE; 258 MAIN AVE</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>MAIN NORWALK LLC; EXPCT LLC; NORTHEAST HOLDINGS ASSOCIATES; HYDE PARK PROPERTIES LLC</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Improved; Commercial Improved; Commercial Vacant; Commercial Improved</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Norwalk</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>*** Main Avenue</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>280 MAIN AVE; 300 MAIN AVE; 306 MAIN AVE; 258 MAIN AVE</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>MAIN NORWALK LLC; EXPCT LLC; NORTHEAST HOLDINGS ASSOCIATES; HYDE PARK PROPERTIES LLC</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Improved; Commercial Improved; Commercial Vacant; Commercial Improved</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>** Bank Street</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>15 BANK STREET; 29 BANK STREET; 25 BANK STREET; 45 BANK STREET</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>15 BANK STREET LLC; BANK 29 LLC; BANK 25 LLC; GNA ASSOCIATES LLC</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>*** First Stamford Place</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>MetroPCS→TMO?, Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="n"/>
+      <c r="H73" s="7" t="n"/>
+      <c r="I73" s="7" t="n"/>
+      <c r="J73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>One Omega Drive</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>in-building IP access</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n"/>
+      <c r="G74" s="7" t="n"/>
+      <c r="H74" s="7" t="n"/>
+      <c r="I74" s="7" t="n"/>
+      <c r="J74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>*** Main Street</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>207 MAIN STREET; 247 MAIN STREET; 239 MAIN STREET; 219 MAIN STREET</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>TM REALTY ASSOCIATES LLC; ROMANO BROTHERS LLC; ROMANO BROTHERS LLC; 219 MAIN STREET LLC</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>*** High Ridge Road</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>908 HIGH RIDGE ROAD; 868 HIGH RIDGE ROAD; 996 HIGH RIDGE ROAD; 878 HIGH RIDGE ROAD</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>HIGH RIDGE REAL ESTATE LLC; 868 HIGH RIDGE ROAD LLC; STAMFORD FOUR LLC; SOUTHERN NEW ENGLAND TELE CO</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Industrial  MDL-94</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>**** Washington Boulevard</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>1351 WASHINGTON BOULEVARD; 1231 WASHINGTON BOULEVARD; 1455 WASHINGTON BOULEVARD; 1315 WASHINGTON BOULEVARD</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>80 WEP-1351 LLC 50% ET AL; PARISH ST ANDREWS PRO EP CH; STAMCON HOLDINGS LLC; GARDEN HOMES STANLEY COURT LTD PTNSHP</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Exmpt Comm  MDL-94; Apartment  MDL-94; Apartment  MDL-94</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>** Strawberry Hill Avenue</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>26 STRAWBERRY HILL AVENUE; 55 STRAWBERRY HILL AVENUE; 44 STRAWBERRY HILL AVENUE; 44 STRAWBERRY HILL AVENUE</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>STAMFORD STRAWBRY HILL ASSOC; TOWN OF STAMFORD; GHORBANIPARVAR MOHAMMADREA; GHORBANIPARVAR MOHAMMADREA</t>
+        </is>
+      </c>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>Apartment  MDL-94; Exmpt Comm  MDL-94; Comm Condo  MDL-06; Comm Condo  MDL-06</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="n">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>**** Summer Street</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>MetroPCS→TMO?</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>2720 SUMMER STREET; 1959 SUMMER STREET; 2802 SUMMER STREET; 1290 SUMMER STREET</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>2720 SUMMER LLC; SMITH JASON; R M E  ASSOCIATES; JENN REALTY LLC</t>
+        </is>
+      </c>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="n">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>* Metro Center (* Station Place)</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>Nextel→TMO?, Sprint→TMO?</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="n"/>
+      <c r="H80" s="7" t="n"/>
+      <c r="I80" s="7" t="n"/>
+      <c r="J80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>**** Washington Blvd</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Verizon</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>1351 WASHINGTON BOULEVARD; 1231 WASHINGTON BOULEVARD; 1455 WASHINGTON BOULEVARD; 1315 WASHINGTON BOULEVARD</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>80 WEP-1351 LLC 50% ET AL; PARISH ST ANDREWS PRO EP CH; STAMCON HOLDINGS LLC; GARDEN HOMES STANLEY COURT LTD PTNSHP</t>
+        </is>
+      </c>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Exmpt Comm  MDL-94; Apartment  MDL-94; Apartment  MDL-94</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>*** Long Ridge Road</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>in-building IP access</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>T-Mobile</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>316 LONG RIDGE ROAD; 961 LONG RIDGE ROAD; 295 LONG RIDGE ROAD; 900 LONG RIDGE ROAD</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>DAGOSTINO JOSEPH ET AL; HORN &amp; HOOF PROPERTIES LLC; WED US LLC; 900 LONG RIDGE ROAD PROPERTY OWNER LLC</t>
+        </is>
+      </c>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94; Commercial  MDL-94</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Stamford</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>** Station Place</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>rooftop</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>AT&amp;T</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="7" t="n"/>
+      <c r="H83" s="7" t="n"/>
+      <c r="I83" s="7" t="n"/>
+      <c r="J83" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J23"/>
+  <autoFilter ref="A4:J83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add owner mailing address + last sale date/price to lead output
Pulls three fields from each candidate parcel's raw CAMA row:
  Owner Mailing Address <- mailing_address(+_2)/city/state/zip
  Last Sale Date        <- sale_date
  Last Sale Price       <- sale_price
Values align 1:1 with the candidate parcel list.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eb8pFNbEASzxnuWc7CqGLH
</commit_message>
<xml_diff>
--- a/cttowerleads/ct-tower-leads/output/leads.xlsx
+++ b/cttowerleads/ct-tower-leads/output/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$4:$J$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$4:$M$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -479,8 +479,11 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,10 +543,25 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>Owner Mailing Address</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Last Sale Date</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Last Sale Price</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
           <t>Use</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t># Cands</t>
         </is>
@@ -586,10 +604,25 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
+          <t>105 BLOOMFIELD AV, HARTFORD CT 06105-1008; 111 BLOOMFIELD AVE, HARTFORD CT 06105; 111 BLOOMFIELD AVE, HARTFORD CT 06105; 145 BLOOMFIELD AV, HARTFORD CT 06105-1008</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>8/25/2000; 11/27/2019; 11/27/2019; —</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>$662,000; $0; $0; —</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
           <t>ONE FAMILY; VAC UNDV RES; VAC LAND RES; AUX IMP RES</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>38</v>
       </c>
     </row>
@@ -634,10 +667,25 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
+          <t>9 FARM SPRING RD, C/O HARTFORD HEALTHCARE CORP. TAX DEPARTMENT, FARMINGTON CT 06032-3315; 9 FARM SPRING RD, C/O HARTFORD HEALTHCARE CORP. TAX DEPARTMENT, FARMINGTON CT 06032-3315; 1 BUCKHEAD PLAZA, 3060 PEACHTREE RD NW STE 1030, ATLANTA GA 30305; 80 SEYMOUR ST, HARTFORD CT 06102-8000</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>5/7/2009; 5/2/2007; 11/3/2021; 6/17/2002</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>$250,000; $520,000; —; $15,028,598</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
           <t>MED OFFICE; MED OFFICE; MED OFFICE; GEN HOSPITAL</t>
         </is>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -682,10 +730,25 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
+          <t>783 EAST MAIN ST, MERIDEN CT 06450; 241 TALCOTT NOTCH RD, FARMINGTON CT 06032; 6 FIRETHORN DR, EDISON NJ 08820; 113 EAST MAIN ST, MERIDEN CT 06450</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>—; 8/8/2016; 8/31/2021; 11/1/2023</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>—; $0; $1,260,000; $375,000</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Apt</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>181</v>
       </c>
     </row>
@@ -730,10 +793,25 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
+          <t>315 PECK ST, NEW HAVEN CT 06513; PO BOX 16534, WEST HAVEN CT 06516; 106 PECK ST, NEW HAVEN CT 06513; 102 PECK ST, NEW HAVEN CT 06513</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>5/31/2002; 2/8/2022; 10/31/2011; 7/31/2002</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>$2,400,000; $0; $170,000; $0</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
           <t>INDUSTRIAL  MDL-96; Three Family; Two Family; Three Family</t>
         </is>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>64</v>
       </c>
     </row>
@@ -774,10 +852,25 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
+          <t>72 CHAPEL STREET, DERBY CT 06418; PO BOX 268, WEST HAVEN CT 06516; 300 WHALLEY AV, NEW HAVEN CT 06511; 1605 WHALLEY AVE, NEW HAVEN CT 06515</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>12/21/2011; 2/24/1989; 2/22/1994; 2/23/2015</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $0</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
           <t>COMM WHSE  MDL-95; OFFICE BLD  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>296</v>
       </c>
     </row>
@@ -822,10 +915,25 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
+          <t>2175 HUDSON TER, FORT LEE NJ 07024-0000; ATTN CLAYTON ROESCH, 803 STANLEY AVENUE, PENSACOLA FL 32503; 1400 OLD COUNTRY RD, WESTBURY NY 11590-0000; 185 N W SPANISH RIVER BLVD SUITE 100, BOCA RATON FL 33431-0000</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>6/7/2021; 3/3/1992; 11/5/2019; 8/16/2019</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>$22,900,000; $0; $15,000,000; $0</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
           <t>Apartments - Com; Commercial Improved; Commercial Improved; Commercial Improved</t>
         </is>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>69</v>
       </c>
     </row>
@@ -870,10 +978,25 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
+          <t>25 BELDEN AVE, NORWALK CT 06850-3303; 125 EAST AVENUE, NORWALK CT 06851; 4040 WILSON BLVD STE 1000, ARLINGTON VA 22203; 80 CUTTER MILL RD., SUITE 411, GREAT NECK NY 11021</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>12/30/1988; 1/29/2024; 8/11/1997; 9/17/1998</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>$0; $800,000; $0; $0</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
           <t>Commercial Improved; Commercial Improved; Commercial Improved; Commercial Improved</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>12</v>
       </c>
     </row>
@@ -906,6 +1029,9 @@
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -948,10 +1074,25 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
+          <t>1 LANDMARK SQ STE 220, STAMFORD CT 06901-; 1 TOWER SQ MS 1, ATTN: THOMAS M. LUSZCZAK, HARTFORD CT 06183-0001; PO BOX 270, HARTFORD CT 06141-0270; 384 OLD TURNPIKE RD, SOUTHINGTON CT 06489</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>12/4/2023; 3/19/2002; —; 3/8/2019</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>$3,820,000; $10; —; $325,000</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
           <t>GEN OFFICE; GEN OFFICE; AUX IMP COMM; GEN OFFICE</t>
         </is>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="M13" s="6" t="n">
         <v>52</v>
       </c>
     </row>
@@ -996,10 +1137,25 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
+          <t>450 CAPITOL AV MS 55FIN, C/O OFFICE OF POLICY &amp; MANAGEMENT, HARTFORD CT 06106-1365; PO BOX 548, PORTLAND CT 06480-0548; 70 FARM VIEW DR, c/o Utility Shared Services-Local Tax, NEW GLOUCESTER ME 04260-5118; 60 COLUMBUS BLVD, HARTFORD CT 06103-2805</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>2/15/2001; 2/16/2007; —; —</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>$0; $1,600,000; —; —</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
           <t>ST-ADMINISTR; HIGH RISE OF; OTHER UTILTY; A PARKING</t>
         </is>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="M14" s="6" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1044,10 +1200,25 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
+          <t>30 PINERIDGE DR EXT, WATERTOWN CT 06779; 144 LEWIS AVE, MERIDEN CT 06451; 25 BROWNSTONE RD, BERLIN CT 06037; 150 GREAT NECK RD  STE 304, GREAT NECK NY 11021</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>6/24/2021; 11/8/2012; 2/26/2019; 6/8/2020</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>$1; $190,000; $0; $12,500,000</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Land</t>
         </is>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="M15" s="6" t="n">
         <v>61</v>
       </c>
     </row>
@@ -1088,10 +1259,25 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
+          <t>410 2ND AVE, WEST HAVEN CT 06516; 99 SHELTON AV, NEW HAVEN CT 06511; 91 SHELTON AV, NEW HAVEN CT 06511; 5010 WHEELER RD, OXON HILL MD 20745</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>5/13/2016; 10/14/2008; 5/17/2005; 11/1/2012</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>$75,000; $675,000; $0; $45,000</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; INDUSTRIAL  MDL-96; INDUSTRIAL  MDL-96; Two Family</t>
         </is>
       </c>
-      <c r="J16" s="6" t="n">
+      <c r="M16" s="6" t="n">
         <v>147</v>
       </c>
     </row>
@@ -1136,10 +1322,25 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
+          <t>433 TEMPLE ST, NEW HAVEN CT 06511; 29 PLATT AV, WEST HAVEN CT 06516; 648 PROSPECT ST, NEW HAVEN CT 06511; YALE U CONTROLLER FRA, PO BOX 208372, NEW HAVEN CT 06520-8372</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>8/4/2023; 8/20/2007; 7/3/2018; 5/18/1990</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>$2,850,000; $0; $0; $0</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
           <t>OFFICE BLD  MDL-94; APT5 - 12 R  MDL-03; Single Family; PVT UNIV  MDL-94</t>
         </is>
       </c>
-      <c r="J17" s="6" t="n">
+      <c r="M17" s="6" t="n">
         <v>59</v>
       </c>
     </row>
@@ -1180,10 +1381,25 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
+          <t>1190 WHALLEY AV, NEW HAVEN CT 06515; 1297 WHALLEY AVE., NEW HAVEN CT 06511; 4066 WHITNEY AV, HAMDEN CT 06518; 1045 WHALLEY AV, NEW HAVEN CT 06511</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>6/17/1996; 3/17/1997; 12/3/2008; 12/22/2009</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>$0; $123,666; $330,000; $230,000</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; OFFICE BLD  MDL-94</t>
         </is>
       </c>
-      <c r="J18" s="6" t="n">
+      <c r="M18" s="6" t="n">
         <v>296</v>
       </c>
     </row>
@@ -1224,10 +1440,25 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
+          <t>178 CHAPEL ST, NEW HAVEN CT 06511; 770 5TH AVENUE, BROOKLYN NY 11232; 565 ELLSWORTH AVE, NEW HAVEN CT 06511; PO BOX 936, MONSEY NY 10952</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>6/26/2009; 2/1/2019; 2/24/2023; 10/30/2020</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>$290,000; $640,000; $265,000; $0</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
           <t>INDUSTRIAL  MDL-96; INDUSTRIAL  MDL-96; COMM WHSE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J19" s="6" t="n">
+      <c r="M19" s="6" t="n">
         <v>402</v>
       </c>
     </row>
@@ -1268,10 +1499,25 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 32547, CHARLOTTE NC 28232; 255 BEAR HILL RD  STE  101, WALTHAM MA 02451; 355 WEST MAIN STREET, STAMFORD CT 06902; 55-15 43RD STREET, MASPETH NY 11378-2023</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>3/12/1997; 2/7/2002; 12/24/2003; 6/30/2017</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>$0; $350,000; $85,000; $1,500,000</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94; Commercial  MDL-00</t>
         </is>
       </c>
-      <c r="J20" s="6" t="n">
+      <c r="M20" s="6" t="n">
         <v>141</v>
       </c>
     </row>
@@ -1312,10 +1558,25 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
+          <t>22 KNAPP STREET, STAMFORD CT 06907-1700; P O BOX 4401, STAMFORD CT 06907-0401; 70 KNAPP ST, STAMFORD CT 06907-1728; 88 KNAPP STREET, STAMFORD CT 06907-1730</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>8/4/2021; 3/8/1978; 4/15/2002; 8/19/2020</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>$1,175,000; $0; $0; $515,000</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Apartment  MDL-94; Single Family; Single Family</t>
         </is>
       </c>
-      <c r="J21" s="6" t="n">
+      <c r="M21" s="6" t="n">
         <v>31</v>
       </c>
     </row>
@@ -1360,10 +1621,25 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 3281, STAMFORD CT 06905; PO BOX 110472, STAMFORD CT 06911; 42 HEDGE BROOK LANE, STAMFORD CT 06903-2029; 61 SEAVIEW AVENUE #66, STAMFORD CT 06902-6042</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>12/30/1992; 3/16/2000; 5/11/2018; 4/21/2022</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $850,000; $412,000</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
           <t>Apartment  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Res. Condo</t>
         </is>
       </c>
-      <c r="J22" s="6" t="n">
+      <c r="M22" s="6" t="n">
         <v>85</v>
       </c>
     </row>
@@ -1404,10 +1680,25 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
+          <t>38 ELM ST, MERIDEN CT 06450; 60-06 39TH AVE, WOODSIDE NY 11377; 7 MAJESTIC CT, DIX HILLS NY 11746; 80 ELM ST, MERIDEN CT 06450</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>—; 4/11/2022; 2/3/2020; 5/29/2019</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>—; $877,500; $320,000; $100,000</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Ind Bldg; Res Impr; Res Impr</t>
         </is>
       </c>
-      <c r="J23" s="6" t="n">
+      <c r="M23" s="6" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1448,10 +1739,25 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
+          <t>750 WORDIN AVE, BRIDGEPORT CT 06605; 60 WASHINGTON ST, HARTFORD CT 06106; 129 WORDIN AVE, BRIDGEPORT CT 06606; 701 WESTERN AVENUE, GLENDALE CA 91201-5025</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>1/6/1987; 2/14/1974; 3/5/2012; 6/30/1989</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $5,076,000</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
           <t>Industrial Mdl 96; Industrial Lnd; Industrial Mdl 96; Self Storage</t>
         </is>
       </c>
-      <c r="J24" s="6" t="n">
+      <c r="M24" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1492,10 +1798,25 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
+          <t>336 DOVER ST, BRIDGEPORT CT 06610; 77 LANSBURY ROAD, TRUMBULL CT 06611; 138 ARCTIC ST, BRIDGEPORT CT 06608-1826; 265 HARVEST RIDGE RD, STRATFORD CT 06614</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>11/18/2019; 11/24/2008; 7/7/2021; 3/3/2004</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>$85,500; $56,500; $0; $0</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
           <t>Two Family; Single Family; Single Family; Two Family</t>
         </is>
       </c>
-      <c r="J25" s="6" t="n">
+      <c r="M25" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1540,10 +1861,25 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
+          <t>P O BOX 55416, BRIDGEPORT CT 06610; 114  ALBEMARLE  RD  APT B4, BROOKLYN NY 11218; 2316 79TH STREET, BROOKLYN NY 11214; 17 WOODBINE ROAD, WOODBRIDGE CT 06525</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>7/26/2012; 8/5/2002; 8/5/2002; 6/30/2009</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>$540,000; $620,000; $620,000; $275,000</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
           <t>Mix Use Comm; Comm Apts; Mix Use Comm; Comm Apts</t>
         </is>
       </c>
-      <c r="J26" s="6" t="n">
+      <c r="M26" s="6" t="n">
         <v>149</v>
       </c>
     </row>
@@ -1588,10 +1924,25 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 6214, BRIDGEPORT CT 06606; 25 GREENLAWN DR, FAIRFIELD CT 06825; 448 PARK AVE, # 460, BRIDGEPORT CT 06604; 378 PARK AVE, BRIDGEPORT CT 06604</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>9/18/2003; 5/17/2012; 12/28/2005; 3/21/2022</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $700,000; $380,000</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
           <t>Mix Use Comm; Retail Strip/Plaza; Comm Apts; Mix Use Comm</t>
         </is>
       </c>
-      <c r="J27" s="6" t="n">
+      <c r="M27" s="6" t="n">
         <v>265</v>
       </c>
     </row>
@@ -1636,10 +1987,25 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
+          <t>61 INTERSTATE LANE, WATERBURY CT 06705; 53 HARDESTY RD, STAMFORD CT 06903; 789 HOWARD AVE, MCS-2 ATTN:  TAX DEPARTMENT, NEW HAVEN CT 06519; 789 HOWARD AVENUE, MCS-2 ATTN:  TAX DEPARTMENT, NEW HAVEN CT 06519</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>2/24/2017; 1/25/2002; 1/1/2000; 1/1/2000</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>$320,000; $225,000; $0; $0</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
           <t>Industrial Mdl 96; Industrial Mdl 96; Hospital; Hospital</t>
         </is>
       </c>
-      <c r="J28" s="6" t="n">
+      <c r="M28" s="6" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1680,10 +2046,25 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
+          <t>381 HIGHLAND AVE, WEST HAVEN CT 06816; 125 ALBRIGHT AVE, STRATFORD CT 06614; 8723 BALMORAL DRIVE, NEWCASTLE CA 95658; 70 EDWARD ST, WEST HAVEN CT 06516</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>4/11/2002; 10/5/2018; 9/9/2004; 8/17/2000</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>$30,845; $100,000; $265,000; $28,000</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
           <t>Vac Comm Lnd; Mix Use Comm; Comm Apts; Single Family</t>
         </is>
       </c>
-      <c r="J29" s="6" t="n">
+      <c r="M29" s="6" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1716,6 +2097,9 @@
       <c r="H30" s="7" t="n"/>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="6" t="n"/>
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1754,10 +2138,25 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
+          <t>2362 NOSTRAND AVE SUITE 7, BROOKLYN NY 11210; 61 WILLETT ST #A, PASSAIC NJ 07055; 619 EASTERN PKWY, BROOKLYN NY 11213; 550 MAIN ST, HARTFORD CT 06103-2913</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>12/27/2019; 1/11/2017; 1/21/2022; 3/7/2003</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>$3,172,808; $850,000; $1,050,000; $0</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
           <t>GEN OFFICE; RETAIL GEN; GEN OFFICE; CITY-FIRE</t>
         </is>
       </c>
-      <c r="J31" s="6" t="n">
+      <c r="M31" s="6" t="n">
         <v>280</v>
       </c>
     </row>
@@ -1798,10 +2197,25 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
+          <t>75 COLUMBIA AVENUE, C/O NATIONWIDE POSTAL MGMT., CEDARHURST NY 11516-2302; 46 CENTER SQUARE, EAST LONGMEADOW MA 01028; 92 HILLDALE RD, WEST HARTFORD CT 06117-1413; 39 SUMMIT DR, WINDSOR CT 06095-3238</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>—; 7/13/2015; 5/31/2016; 12/19/2008</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>—; $20,750,000; $0; $0</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
           <t>GEN OFFICE; MED OFFICE; RETAIL GEN; APARTMENT</t>
         </is>
       </c>
-      <c r="J32" s="6" t="n">
+      <c r="M32" s="6" t="n">
         <v>68</v>
       </c>
     </row>
@@ -1842,10 +2256,25 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 876, ITHACA NY 14851-0876; PO BOX 876, ITHACA NY 14851-0876; 300 SUMMIT ST, HARTFORD CT 06106-3100; 453 SUMMIT ST, HARTFORD CT 06106-2354</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>6/8/1998; 6/8/1998; 12/10/2001; 2/1/2000</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $82,000</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
           <t>CHARITABLE; HALL - CLUB; PRIV COLLEGE; THREE FAMILY</t>
         </is>
       </c>
-      <c r="J33" s="6" t="n">
+      <c r="M33" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1886,10 +2315,25 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
+          <t>8101  RICHARDSON RD STE 101, COMMERCE TWP MI 06416; 2800 BERLIN TPKE, NEWINGTON CT 06111-4113; 2800 BERLIN TPKE, NEWINGTON CT 06111-4113; 545 BROADWAY 4TH FLOOR, c/o CARNEGIE MANAGEMENT, BROOKLYN NY 11206</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>2/24/2020; 8/6/2008; —; 8/16/2021</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; —; $3,700,000</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
           <t>HIGH RISE OF; ST-DOT; ST-MISC PROP; HIGH RISE OF</t>
         </is>
       </c>
-      <c r="J34" s="6" t="n">
+      <c r="M34" s="6" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1930,10 +2374,25 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
+          <t>2362 NOSTRAND AVE SUITE 7, BROOKLYN NY 11210; 1608 WALNUT ST, SUITE 1400, C/O ROBERT WEINSTEIN, PHILADELPHIA PA 19103; 36 TRUMBULL ST, HARTFORD CT 06103-2404; 2362 NOSTRAND AVE STE 7, BROOKLYN NY 11210-</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>8/3/2021; 2/19/2003; 7/30/2013; 6/27/2023</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>$2,350,000; $2,400,000; $0; $4,750,000</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
           <t>GEN OFFICE; APT HIGH RSE; GEN OFFICE; HIGH RISE OF</t>
         </is>
       </c>
-      <c r="J35" s="6" t="n">
+      <c r="M35" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1978,10 +2437,25 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
+          <t>3000 WHITNEY AVE 299, HAMDEN CT 06518-; 132 PRESTON ST, WINDSOR CT 06095-3135; 97 LEVERICH DR, EAST HARTFORD CT 06108-1432; 2281 MAIN ST, HARTFORD CT 06120-2022</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>7/14/2023; —; 11/7/2005; 5/29/2007</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>$560,000; —; $183,000; $300,000</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
           <t>APART/COMM; RETAIL GEN; RES/COMM; RES/COMM</t>
         </is>
       </c>
-      <c r="J36" s="6" t="n">
+      <c r="M36" s="6" t="n">
         <v>280</v>
       </c>
     </row>
@@ -2022,10 +2496,25 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
+          <t>2800 BERLIN TPKE, NEWINGTON CT 06111-4113; PO BOX 317546, NEWINGTON CT 06131-7546; 505 8TH AV 15FL, C/O COMMON GROUND, NEW YORK NY 10018-4531; 1 MONARCH PL, SPRINGFIELD MA 01144-1099</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>—; —; 9/23/2003; 2/3/1999</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>—; —; $0; $0</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
           <t>ST-MISC PROP; ST-HWY PROP; APART/COMM; L PARKING</t>
         </is>
       </c>
-      <c r="J37" s="6" t="n">
+      <c r="M37" s="6" t="n">
         <v>28</v>
       </c>
     </row>
@@ -2066,10 +2555,25 @@
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
+          <t>246 MARKET ST SUITE 332, PATERSON NJ 07505; 112 PROSPECT AV, HARTFORD CT 06106-2956; 1429 PARK ST SUITE 205, HARTFORD CT 06106-2051; 62 RAMHORNE RD, NEW CANAAN CT 06840</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>1/24/2022; 12/30/2008; 1/19/2006; 10/21/2021</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>$4,220,000; $0; $0; $1,850,000</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
           <t>APARTMENT; GEN OFFICE; RETAIL GEN; APARTMENT</t>
         </is>
       </c>
-      <c r="J38" s="6" t="n">
+      <c r="M38" s="6" t="n">
         <v>124</v>
       </c>
     </row>
@@ -2110,10 +2614,25 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
+          <t>356 FREEMAN ST, HARTFORD CT 06106; 137 SISSON AV, HARTFORD CT 06105; 48 WEST 38TH ST 10TH FLOOR, NEW YORK NY 10018; 99 SISSON AV, HARTFORD CT 06106-1131</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>4/2/2003; 1/31/2013; 6/7/2021; 11/21/2003</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>$0; $424,000; $741,000; $1</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
           <t>RES/COMM; RETAIL GEN; APARTMENT; APART/COMM</t>
         </is>
       </c>
-      <c r="J39" s="6" t="n">
+      <c r="M39" s="6" t="n">
         <v>76</v>
       </c>
     </row>
@@ -2154,10 +2673,25 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
+          <t>C/O STATE-MARKET HARTFORD LLC, 90 STATE ST - MGT OFFICE, HARTFORD CT 06103; C/O STATE-MARKET HARTFORD LLC, 90 STATE ST - MGT OFFICE, HARTFORD CT 06103; C/O STATE-MARKET HARTFORD LLC, 90 STATE ST - MGT OFFICE, HARTFORD CT 06103; 90 STATE HOUSE SQUARE, c/o STATE MARKET HARTFORD LLC, HARTFORD CT 06103</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>10/14/2003; 10/14/2003; 10/14/2003; 2/28/2007</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $97,750,000</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
           <t>VAC LAND COM; VAC LAND COM; VAC LAND COM; HIGH RISE OF</t>
         </is>
       </c>
-      <c r="J40" s="6" t="n">
+      <c r="M40" s="6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2198,10 +2732,25 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
+          <t>1870 PARK ST, HARTFORD CT 06106-2136; 1835 PARK ST, HARTFORD CT 06106-2121; 1816 PARK ST, HARTFORD CT 06106-2135; 12 SOUTH WHITNEY ST, HARTFORD CT 06106</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>6/16/1999; 12/18/2001; 7/21/2000; 10/2/2014</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>$80,000; $93,100; $40,000; $220,000</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
           <t>RES/COMM; RETAIL GEN; RETAIL GEN; COMM &amp; APART</t>
         </is>
       </c>
-      <c r="J41" s="6" t="n">
+      <c r="M41" s="6" t="n">
         <v>163</v>
       </c>
     </row>
@@ -2242,10 +2791,25 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
+          <t>8 BREWER ST, EAST HARTFORD CT 06118; 135 BROAD ST, HARTFORD CT 06105-3718; ONE HARTFORD PLAZA, ATTN: REAL ESTATE DEPT - TOWER 12, HARTFORD CT 06115; 225 GARDEN ST, HARTFORD CT 06105</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>3/6/2020; 5/12/2008; 7/3/2008; 2/9/2022</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>$350,000; $0; $9,100,000; $1</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
           <t>APARTMENT; CHARITABLE; HIGH RISE OF; ONE FAMILY</t>
         </is>
       </c>
-      <c r="J42" s="6" t="n">
+      <c r="M42" s="6" t="n">
         <v>177</v>
       </c>
     </row>
@@ -2286,10 +2850,25 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
+          <t>136 BARTHOLOMEW AVE, HARTFORD CT 06106; 82-84 FRANCIS AVE, HARTFORD CT 06106; 2074 PARK ST SUITE 101, HARTFORD CT 06106; 190 SHADOW LAKE RD, RIDGEFIELD CT 06877</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>2/21/2023; 5/26/2022; 1/4/2019; 5/17/2021</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>$120,000; $525,000; $550,000; $0</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
           <t>ONE FAMILY; APARTMENT; VAC LAND IND; MANUFACTURNG</t>
         </is>
       </c>
-      <c r="J43" s="6" t="n">
+      <c r="M43" s="6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2330,10 +2909,25 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
+          <t>14 SYCAMORE WAY, WALLINGFORD CT 06492; 901 MAPLE AV, HARTFORD CT 06114-2330; 871 MAPLE AVE, HARTFORD CT 06114; 315 HIGHLAND AVE SUITE 102, CHESHIRE CT 06401</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>6/18/2007; 6/13/2008; 3/11/2013; 10/4/2021</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>$385,000; $0; $400,000; $65,000</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
           <t>AUX IMP COMM; RETAIL GEN; RETAIL GEN; RETAIL GEN</t>
         </is>
       </c>
-      <c r="J44" s="6" t="n">
+      <c r="M44" s="6" t="n">
         <v>143</v>
       </c>
     </row>
@@ -2374,10 +2968,25 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
+          <t>20 OCEAN CT, BROOKLYN NY 11223-6054; 91 NORTHWEST DR, PLAINVILLE CT 06062; 114 WOODLAND ST, HARTFORD CT 06105-1208; 40 WOODLAND ST, HARTFORD CT 06105-2327</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>5/2/2008; 4/2/2019; —; 2/25/2003</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>$0; $1; —; $0</t>
+        </is>
+      </c>
+      <c r="L45" s="7" t="inlineStr">
+        <is>
           <t>MED OFFICE; MED OFFICE; MED OFFICE; GEN OFFICE</t>
         </is>
       </c>
-      <c r="J45" s="6" t="n">
+      <c r="M45" s="6" t="n">
         <v>68</v>
       </c>
     </row>
@@ -2422,10 +3031,25 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
+          <t>501 CHESTNUT RIDGE RD, SPRING VALLEY NY 10977; 25 ALLIK WAY SUITE 536, SPRING VALLEY NY 10977; 97 WEBSTER ST, HARTFORD 06114; 255 HOMESTEAD AVE, HARTFORD CT 06112</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>—; 3/23/2023; 12/4/2019; 2/2/2016</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>—; $2,000,000; $150,000; $141,000</t>
+        </is>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
           <t>APARTMENT; APARTMENT; ONE FAMILY; CHARITABLE</t>
         </is>
       </c>
-      <c r="J46" s="6" t="n">
+      <c r="M46" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2466,10 +3090,25 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
+          <t>86 FARMINGTON AV, C/O BRUCE G MACDERMID, HARTFORD CT 06105-3704; 5111 AVE L, BROOKLYN NY 11234-; 43 CHEPACHET RD, AVON CT 06001; 505 FARMINGTON AV, HARTFORD CT 06105-3105</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>6/25/1999; 2/9/2024; —; —</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>$303,000; $1; —; —</t>
+        </is>
+      </c>
+      <c r="L47" s="7" t="inlineStr">
+        <is>
           <t>GEN OFFICE; APART/COMM; RES/COMM; COMM/RES</t>
         </is>
       </c>
-      <c r="J47" s="6" t="n">
+      <c r="M47" s="6" t="n">
         <v>107</v>
       </c>
     </row>
@@ -2510,10 +3149,25 @@
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
+          <t>1022 BOULEVARD SUITE 183, WEST HARTFORD CT 06119; 15 WEBSTER ST, HARTFORD CT 06114; 105 GARDEN DR APT 2, MANCHESTER NH 03102; 15 WEBSTER ST, HARTFORD CT 06114</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>5/2/2022; 2/14/2022; 9/15/2023; 8/18/2021</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>$8,600,000; $0; $450,000; $0</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
           <t>APARTMENT; APARTMENT; APARTMENT; THREE FAMILY</t>
         </is>
       </c>
-      <c r="J48" s="6" t="n">
+      <c r="M48" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2554,10 +3208,25 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
+          <t>167 BRAINARD RD, HARTFORD CT 06114; 160 BRAINARD RD, HARTFORD CT 06114; 920 S COLONY RD, C/O DEMARTINO FIXTURE CO, INC, WALLINGFORD CT 06492-5263; 555 MAIN ST, HARTFORD CT 06103-2915</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>5/26/2023; 12/14/2009; —; 7/1/2010</t>
+        </is>
+      </c>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>$2,500,000; $840,000; —; $1,600,000</t>
+        </is>
+      </c>
+      <c r="L49" s="7" t="inlineStr">
+        <is>
           <t>RETAIL GEN; RETAIL GEN; RETAIL GEN; SPECIAL ACTS</t>
         </is>
       </c>
-      <c r="J49" s="6" t="n">
+      <c r="M49" s="6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2598,10 +3267,25 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
+          <t>743 ELM ST, ROCKY HILL CT 06067; 200 PRATT ST, MERIDEN CT 06450; P O BOX 9456, MINNEAPOLIS MN 55440; 22 CHURCH ST, MERIDEN CT 06451</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>4/1/2019; —; 1/30/2001; 9/1/2010</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>$273,000; —; $0; $0</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Apt; Comm Bldg; Comm Apt</t>
         </is>
       </c>
-      <c r="J50" s="6" t="n">
+      <c r="M50" s="6" t="n">
         <v>49</v>
       </c>
     </row>
@@ -2646,10 +3330,25 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
+          <t>783 EAST MAIN ST, MERIDEN CT 06450; 241 TALCOTT NOTCH RD, FARMINGTON CT 06032; 6 FIRETHORN DR, EDISON NJ 08820; 113 EAST MAIN ST, MERIDEN CT 06450</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>—; 8/8/2016; 8/31/2021; 11/1/2023</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>—; $0; $1,260,000; $375,000</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Apt</t>
         </is>
       </c>
-      <c r="J51" s="6" t="n">
+      <c r="M51" s="6" t="n">
         <v>181</v>
       </c>
     </row>
@@ -2686,6 +3385,9 @@
       <c r="H52" s="7" t="n"/>
       <c r="I52" s="7" t="n"/>
       <c r="J52" s="6" t="n"/>
+      <c r="K52" s="6" t="n"/>
+      <c r="L52" s="7" t="n"/>
+      <c r="M52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -2728,10 +3430,25 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
+          <t>90 WILLOW ST, MERIDEN CT 06450; 82 WILLOW ST, MERIDEN CT 06450; 230 EAST MAIN ST #3, MERIDEN CT 06450; 24 WILLOW ST, MERIDEN CT 06450</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>10/1/2020; 1/19/2022; 5/9/2005; 12/16/2020</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>$0; $250,000; $25,000; $122,000</t>
+        </is>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Res Impr; Vacant Com; Res Impr</t>
         </is>
       </c>
-      <c r="J53" s="6" t="n">
+      <c r="M53" s="6" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2772,10 +3489,25 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
+          <t>1260 EAST MAIN ST, MERIDEN CT 06450; 234 MIDDLE ST, MIDDLETOWN CT 06457; 170 PRESTON AVE, MERIDEN CT 06450; 66 KINGS HIGHWAY, NORTH HAVEN CT 06473</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>12/28/2006; —; —; 8/10/2022</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>$400,000; —; —; $1,000,000</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Bldg; Comm Bldg; Comm Land</t>
         </is>
       </c>
-      <c r="J54" s="6" t="n">
+      <c r="M54" s="6" t="n">
         <v>181</v>
       </c>
     </row>
@@ -2816,10 +3548,25 @@
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
+          <t>119 SPRUCE ST, MERIDEN CT 06450; 200 PRATT ST, MERIDEN CT 06450; 470 S ELM ST, WALLINGFORD CT 06492; 558 HANOVER ST, MERIDEN CT 06450</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>10/21/2021; —; 5/3/2016; 4/26/2017</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>$325,000; —; $270,000; $0</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
           <t>Comm Bldg; Comm Land; Comm Bldg; Comm Land</t>
         </is>
       </c>
-      <c r="J55" s="6" t="n">
+      <c r="M55" s="6" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2864,10 +3611,25 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
+          <t>P.O BOX 89, THOMASTON CT 06787; 2727 N CENTRAL AVE, PHOENIX AZ 85004; 6 ASPEN DR, MADISON CT 06443; 105 WATER ST, NEW HAVEN CT 06511</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>6/13/1994; 8/18/2016; 8/16/1976; 1/31/2022</t>
+        </is>
+      </c>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>$0; $6,000,000; $0; $1,500,000</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
           <t>INDUSTRIAL  MDL-96; IND WHSES  MDL-96; REST/CLUBS  MDL-94; PARK LOT</t>
         </is>
       </c>
-      <c r="J56" s="6" t="n">
+      <c r="M56" s="6" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2912,10 +3674,25 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
+          <t>541 SHEPARD AVE, HAMDEN CT 06514; YALE U CONTROLLER FRA, PO BOX 208372, NEW HAVEN CT 06520-8372; 3 REDWOOD LANE, WOODBRIDGE CT 06525; 13215 BEE CAVE PKWY, AUSTIN TX 78738</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>4/7/2004; 6/3/2005; 9/15/2011; 11/16/2017</t>
+        </is>
+      </c>
+      <c r="K57" s="6" t="inlineStr">
+        <is>
+          <t>$0; $288,000; $0; $61,252,000</t>
+        </is>
+      </c>
+      <c r="L57" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; HOTELS  MDL-94</t>
         </is>
       </c>
-      <c r="J57" s="6" t="n">
+      <c r="M57" s="6" t="n">
         <v>296</v>
       </c>
     </row>
@@ -2956,10 +3733,25 @@
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
+          <t>90 MCKINLEY AV, NEW HAVEN CT 06511; 84 MCKINLEY AV, NEW HAVEN CT 06515; 76 MCKINLEY AV, NEW HAVEN CT 06515; 70 MCKINLEY AVE, NEW HAVEN CT 06515</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>1/11/2022; 9/11/2015; 7/2/2021; 10/2/1991</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>$570,000; $0; $583,000; $170,000</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
           <t>Single Family; Single Family; Single Family; Single Family</t>
         </is>
       </c>
-      <c r="J58" s="6" t="n">
+      <c r="M58" s="6" t="n">
         <v>82</v>
       </c>
     </row>
@@ -3000,10 +3792,25 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
+          <t>827 ORANGE ST, NEW HAVEN CT 06511; 80 COUNTRY LANE, MILFORD CT 06460; 528 ORANGE ST, NEW HAVEN CT 06511; 494 ORANGE ST, NEW HAVEN CT 06511</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>8/8/2023; 12/13/2017; 11/13/2023; 4/5/2006</t>
+        </is>
+      </c>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $0</t>
+        </is>
+      </c>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J59" s="6" t="n">
+      <c r="M59" s="6" t="n">
         <v>225</v>
       </c>
     </row>
@@ -3044,10 +3851,25 @@
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
+          <t>151 HEMINGWAY AVE, EAST HAVEN CT 06512; 390 WHALLEY AVE, NEW HAVEN CT 06511; PO BOX 936, MONSEY NY 10952; 46-14 UNION ST 1FL, FLUSHING NY 11355</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>4/30/2019; 5/31/2022; 1/28/2020; 3/18/1999</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>$75,000; $0; $0; $278,000</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J60" s="6" t="n">
+      <c r="M60" s="6" t="n">
         <v>234</v>
       </c>
     </row>
@@ -3080,6 +3902,9 @@
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="6" t="n"/>
+      <c r="K61" s="6" t="n"/>
+      <c r="L61" s="7" t="n"/>
+      <c r="M61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -3118,10 +3943,25 @@
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
+          <t>265 COLLEGE ST, NEW HAVEN CT 06510; 75 TUPELO LA, GUILFORD CT 06437; 266 COLLEGE ST, NEW HAVEN CT 06511; YALE U CONTROLLER FRA, PO BOX 208372, NEW HAVEN CT 06520-8372</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>4/18/2022; 11/17/1998; 2/15/2022; 8/4/2004</t>
+        </is>
+      </c>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>$52,500,000; $200,000; $1,700,000; $0</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J62" s="6" t="n">
+      <c r="M62" s="6" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3162,10 +4002,25 @@
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 317546, NEWINGTON CT 06131-7546; 100 POND LILY AV, NEW HAVEN CT 06515; 105 POND LILY AV, NEW HAVEN CT 06515; 111 POND LILY AV, NEW HAVEN CT 06515</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="inlineStr">
+        <is>
+          <t>—; 6/2/2003; 1/6/1998; 11/6/1998</t>
+        </is>
+      </c>
+      <c r="K63" s="6" t="inlineStr">
+        <is>
+          <t>$0; $2,219,000; $101,001; $70,000</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
           <t>STATE DOT  MDL-95; MOTELS; Single Family; Single Family</t>
         </is>
       </c>
-      <c r="J63" s="6" t="n">
+      <c r="M63" s="6" t="n">
         <v>22</v>
       </c>
     </row>
@@ -3198,6 +4053,9 @@
       <c r="H64" s="7" t="n"/>
       <c r="I64" s="7" t="n"/>
       <c r="J64" s="6" t="n"/>
+      <c r="K64" s="6" t="n"/>
+      <c r="L64" s="7" t="n"/>
+      <c r="M64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -3236,10 +4094,25 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
+          <t>399 WHALLEY AV, NEW HAVEN CT 06511; 55 WARREN ST, NEW HAVEN CT 06511; 63 WARREN ST, NEW HAVEN CT 06511; 270 COSEY BEACH AVE, EAST HAVEN CT 06512</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="inlineStr">
+        <is>
+          <t>4/7/2021; 1/10/2020; 9/13/2002; 7/26/2011</t>
+        </is>
+      </c>
+      <c r="K65" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $0; $205,000</t>
+        </is>
+      </c>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
           <t>APT 4-Unit; APT5 - 12  MDL-94; Three Family; Three Family</t>
         </is>
       </c>
-      <c r="J65" s="6" t="n">
+      <c r="M65" s="6" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3280,10 +4153,25 @@
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
+          <t>PO BOX 801, NEW HAVEN CT 06503; 597 WINCHESTER AV, NEW HAVEN CT 06511; 22 LEIGHTON COURT, NORTH HAVEN CT 06473; 520 WINCHESTER AVE, NEW HAVEN CT 06511</t>
+        </is>
+      </c>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>6/7/2004; 3/7/2000; 10/12/2000; 2/5/2019</t>
+        </is>
+      </c>
+      <c r="K66" s="6" t="inlineStr">
+        <is>
+          <t>$0; $79,000; $145,000; $0</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
           <t>INDUSTRIAL  MDL-96; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J66" s="6" t="n">
+      <c r="M66" s="6" t="n">
         <v>176</v>
       </c>
     </row>
@@ -3324,10 +4212,25 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
+          <t>16 SUE TER, WESTPORT CT 06880; 145 OAKLEY ST, NEW HAVEN CT 06513; P.O BOX 8837, NEW HAVEN CT 06532; PO BOX 3060, WESTPORT CT 06880</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>9/21/2020; 7/5/2019; 4/5/2007; 3/28/2005</t>
+        </is>
+      </c>
+      <c r="K67" s="6" t="inlineStr">
+        <is>
+          <t>$762,500; $0; $0; $1,317,500</t>
+        </is>
+      </c>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
           <t>MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94; MIXED USE  MDL-94</t>
         </is>
       </c>
-      <c r="J67" s="6" t="n">
+      <c r="M67" s="6" t="n">
         <v>200</v>
       </c>
     </row>
@@ -3368,10 +4271,25 @@
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
+          <t>2727 N CENTRAL AVE, PHOENIX AZ 85004; 2 SELLECK ST # 3, NORWALK CT 06855-0000; 6 SELLECK ST, NORWALK CT 06855; 90 LEDGEBROOK DR, NORWALK CT 06854</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>6/17/2016; 8/11/1995; 1/16/2014; 10/28/2003</t>
+        </is>
+      </c>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>$4,725,000; $0; $50,000; $375,000</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
           <t>Commercial Improved; 3 Family; Single Family; 2 Family</t>
         </is>
       </c>
-      <c r="J68" s="6" t="n">
+      <c r="M68" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3412,10 +4330,25 @@
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
+          <t>150 PURCHASE ST SUITE 13, RYE NY 10580-0000; 57 WILTON RD, WESTPORT CT 06880-0000; 11 DAY ST, NORWALK CT 06854; ATTN: PATRICK A T LEE, 75 FEDERAL ST SUITE 400, BOSTON MA 02110</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="inlineStr">
+        <is>
+          <t>6/16/2021; 11/20/2019; 8/8/2000; 8/31/2017</t>
+        </is>
+      </c>
+      <c r="K69" s="6" t="inlineStr">
+        <is>
+          <t>$19,900,000; $12,487,400; $0; $0</t>
+        </is>
+      </c>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
           <t>Commercial Improved; Commercial Vacant; Commercial Improved; Apartments - Com</t>
         </is>
       </c>
-      <c r="J69" s="6" t="n">
+      <c r="M69" s="6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3456,10 +4389,25 @@
       </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
+          <t>684 PARK AVE, NEW YORK NY 10065; 8 TWO MILE RD, FARMINGTON CT 06032; 123 HARBOR DR UNIT 211, STAMFORD CT 06902; 258 MAIN AVE, NORWALK CT 06851-2748</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>11/5/2015; 4/3/2007; 3/19/1997; 5/17/2022</t>
+        </is>
+      </c>
+      <c r="K70" s="6" t="inlineStr">
+        <is>
+          <t>$7,995,000; $1,850,000; $1,000,000; $852,500</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
           <t>Commercial Improved; Commercial Improved; Commercial Vacant; Commercial Improved</t>
         </is>
       </c>
-      <c r="J70" s="6" t="n">
+      <c r="M70" s="6" t="n">
         <v>119</v>
       </c>
     </row>
@@ -3500,10 +4448,25 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
+          <t>684 PARK AVE, NEW YORK NY 10065; 8 TWO MILE RD, FARMINGTON CT 06032; 123 HARBOR DR UNIT 211, STAMFORD CT 06902; 258 MAIN AVE, NORWALK CT 06851-2748</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>11/5/2015; 4/3/2007; 3/19/1997; 5/17/2022</t>
+        </is>
+      </c>
+      <c r="K71" s="6" t="inlineStr">
+        <is>
+          <t>$7,995,000; $1,850,000; $1,000,000; $852,500</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
           <t>Commercial Improved; Commercial Improved; Commercial Vacant; Commercial Improved</t>
         </is>
       </c>
-      <c r="J71" s="6" t="n">
+      <c r="M71" s="6" t="n">
         <v>119</v>
       </c>
     </row>
@@ -3544,10 +4507,25 @@
       </c>
       <c r="I72" s="7" t="inlineStr">
         <is>
+          <t>237 MAMARONECK AVENUE, WHITE PLAINS NY 10605; 237 MAMARONECK AVENUE, WHITE PLAINS NY 10605-1319; 237 MAMARONECK AVENUE, WHITE PLAINS NY 10605; 51 BANK STREET, STAMFORD CT 06901</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr">
+        <is>
+          <t>8/28/1998; 5/28/2021; 12/27/2017; 3/15/1995</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>$1,375,000; $1,000,000; $920,000; $300,000</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94</t>
         </is>
       </c>
-      <c r="J72" s="6" t="n">
+      <c r="M72" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3584,6 +4562,9 @@
       <c r="H73" s="7" t="n"/>
       <c r="I73" s="7" t="n"/>
       <c r="J73" s="6" t="n"/>
+      <c r="K73" s="6" t="n"/>
+      <c r="L73" s="7" t="n"/>
+      <c r="M73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -3614,6 +4595,9 @@
       <c r="H74" s="7" t="n"/>
       <c r="I74" s="7" t="n"/>
       <c r="J74" s="6" t="n"/>
+      <c r="K74" s="6" t="n"/>
+      <c r="L74" s="7" t="n"/>
+      <c r="M74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -3652,10 +4636,25 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
+          <t>207 MAIN STREET, STAMFORD CT 06907; 167 GROVE STREET UT I, STAMFORD CT 06901; 167 GROVE STREET UNIT I, STAMFORD CT 06901-1839; P. O. BOX 37214, CHARLOTTE NC 28237</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>2/1/2005; 5/22/2006; 4/24/2017; 9/8/2003</t>
+        </is>
+      </c>
+      <c r="K75" s="6" t="inlineStr">
+        <is>
+          <t>$0; $1,347,880; $2,100,000; $650,000</t>
+        </is>
+      </c>
+      <c r="L75" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94</t>
         </is>
       </c>
-      <c r="J75" s="6" t="n">
+      <c r="M75" s="6" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3696,10 +4695,25 @@
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
+          <t>910 HIGH RIDGE ROAD, STAMFORD CT 06905; 868 HIGH RIDGE ROAD, STAMFORD CT 06905-1911; 460 COE AVENUE, EAST HAVEN CT 06512; PO BOX 2629, ADDISON TX 75001</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="inlineStr">
+        <is>
+          <t>9/30/2008; 8/15/2012; 3/25/2003; 9/14/1976</t>
+        </is>
+      </c>
+      <c r="K76" s="6" t="inlineStr">
+        <is>
+          <t>$1,150,000; $0; $0; $0</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Industrial  MDL-94</t>
         </is>
       </c>
-      <c r="J76" s="6" t="n">
+      <c r="M76" s="6" t="n">
         <v>375</v>
       </c>
     </row>
@@ -3740,10 +4754,25 @@
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
+          <t>333 NORTH BEDFORD ROAD STE 145, MOUNT KISKO NY 10549-1160; 1231 WASHINGTON BLVD, STAMFORD CT 06902-0000; 1920 DEER PARK AVE STE 102, DEER PARK NY 11729-3314; 29 KNAPP STREET, STAMFORD CT 06907-1725</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="inlineStr">
+        <is>
+          <t>9/30/2008; 2/4/1970; 3/18/2019; 1/18/2017</t>
+        </is>
+      </c>
+      <c r="K77" s="6" t="inlineStr">
+        <is>
+          <t>$25,000,000; $0; $60,000,000; $1,325,000</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Exmpt Comm  MDL-94; Apartment  MDL-94; Apartment  MDL-94</t>
         </is>
       </c>
-      <c r="J77" s="6" t="n">
+      <c r="M77" s="6" t="n">
         <v>163</v>
       </c>
     </row>
@@ -3784,10 +4813,25 @@
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
+          <t>234 EAST 40TH ST, NEW YORK NY 10016-1707; 888 WASHINGTON BLVD, STAMFORD CT 06901-2930; 44 STRAWBERRY HILL AVE STE 9, STAMFORD CT 06902-2632; 44 STRAWBERRY HILL AVE STE 9, STAMFORD CT 06902-2632</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="inlineStr">
+        <is>
+          <t>10/18/1971; 1/1/1900; 4/1/2021; 4/1/2021</t>
+        </is>
+      </c>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>$0; $0; $146,875; $103,125</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
           <t>Apartment  MDL-94; Exmpt Comm  MDL-94; Comm Condo  MDL-06; Comm Condo  MDL-06</t>
         </is>
       </c>
-      <c r="J78" s="6" t="n">
+      <c r="M78" s="6" t="n">
         <v>1276</v>
       </c>
     </row>
@@ -3832,10 +4876,25 @@
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
+          <t>15 SQUARE ACRE DRIVE, STAMFORD CT 06905; PO BOX 1769, SILVERTHORNE CO 80498-1769; 121 ST CHARLES AVE, STAMFORD CT 06907-2417; 440 MAMARONECK AVE STE S512, HARRISON NY 10528-2418</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>5/29/2015; 10/9/2019; 9/17/1984; 10/30/2015</t>
+        </is>
+      </c>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>$1,210,000; $0; $0; $12,000,000</t>
+        </is>
+      </c>
+      <c r="L79" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94; Commercial  MDL-94</t>
         </is>
       </c>
-      <c r="J79" s="6" t="n">
+      <c r="M79" s="6" t="n">
         <v>576</v>
       </c>
     </row>
@@ -3872,6 +4931,9 @@
       <c r="H80" s="7" t="n"/>
       <c r="I80" s="7" t="n"/>
       <c r="J80" s="6" t="n"/>
+      <c r="K80" s="6" t="n"/>
+      <c r="L80" s="7" t="n"/>
+      <c r="M80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -3910,10 +4972,25 @@
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
+          <t>333 NORTH BEDFORD ROAD STE 145, MOUNT KISKO NY 10549-1160; 1231 WASHINGTON BLVD, STAMFORD CT 06902-0000; 1920 DEER PARK AVE STE 102, DEER PARK NY 11729-3314; 29 KNAPP STREET, STAMFORD CT 06907-1725</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>9/30/2008; 2/4/1970; 3/18/2019; 1/18/2017</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>$25,000,000; $0; $60,000,000; $1,325,000</t>
+        </is>
+      </c>
+      <c r="L81" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Exmpt Comm  MDL-94; Apartment  MDL-94; Apartment  MDL-94</t>
         </is>
       </c>
-      <c r="J81" s="6" t="n">
+      <c r="M81" s="6" t="n">
         <v>163</v>
       </c>
     </row>
@@ -3954,10 +5031,25 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
+          <t>316 LONG RIDGE RD, STAMFORD CT 06902-1628; 76 NEW CANAAN AVENUE # 7, NORWALK CT 06850-2646; 1297 LONG RIDGE ROAD, STAMFORD CT 06903; 595 MADISON AVE SUITE 1903, NEW YORK NY 10022</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>2/20/1986; 5/7/2018; 3/5/2014; 11/23/2020</t>
+        </is>
+      </c>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>$0; $650,000; $1,000,000; $27,250,000</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
           <t>Commercial  MDL-94; Commercial  MDL-00; Commercial  MDL-94; Commercial  MDL-94</t>
         </is>
       </c>
-      <c r="J82" s="6" t="n">
+      <c r="M82" s="6" t="n">
         <v>265</v>
       </c>
     </row>
@@ -3990,9 +5082,12 @@
       <c r="H83" s="7" t="n"/>
       <c r="I83" s="7" t="n"/>
       <c r="J83" s="6" t="n"/>
+      <c r="K83" s="6" t="n"/>
+      <c r="L83" s="7" t="n"/>
+      <c r="M83" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J83"/>
+  <autoFilter ref="A4:M83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>